<commit_message>
DP: start new future - join_forecast_iplan_230711 - change paths
</commit_message>
<xml_diff>
--- a/create_forecast_basic/future/מיקום מקורי של הקבצים.xlsx
+++ b/create_forecast_basic/future/מיקום מקורי של הקבצים.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="116">
   <si>
     <t>שם קובץ</t>
   </si>
@@ -1155,6 +1155,12 @@
   <si>
     <t>work_factor_230719</t>
   </si>
+  <si>
+    <t>join_forecast_iplan_230711.ipynb</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\iplan\join_forecast</t>
+  </si>
 </sst>
 </file>
 
@@ -1193,7 +1199,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1214,10 +1220,6 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -4564,13 +4566,13 @@
       <c r="Z94" s="2"/>
     </row>
     <row r="95" ht="14.25" customHeight="1">
-      <c r="A95" s="6" t="s">
+      <c r="A95" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B95" s="7" t="s">
+      <c r="B95" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C95" s="6" t="s">
+      <c r="C95" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D95" s="2"/>
@@ -4598,13 +4600,13 @@
       <c r="Z95" s="2"/>
     </row>
     <row r="96" ht="14.25" customHeight="1">
-      <c r="A96" s="6" t="s">
+      <c r="A96" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B96" s="7" t="s">
+      <c r="B96" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C96" s="6" t="s">
+      <c r="C96" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D96" s="2"/>
@@ -4632,13 +4634,13 @@
       <c r="Z96" s="2"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
-      <c r="A97" s="6" t="s">
+      <c r="A97" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B97" s="7" t="s">
+      <c r="B97" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C97" s="6" t="s">
+      <c r="C97" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D97" s="2"/>
@@ -4666,13 +4668,13 @@
       <c r="Z97" s="2"/>
     </row>
     <row r="98" ht="14.25" customHeight="1">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B98" s="7" t="s">
+      <c r="B98" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C98" s="6" t="s">
+      <c r="C98" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D98" s="2"/>
@@ -4700,13 +4702,13 @@
       <c r="Z98" s="2"/>
     </row>
     <row r="99" ht="14.25" customHeight="1">
-      <c r="A99" s="6" t="s">
+      <c r="A99" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B99" s="7" t="s">
+      <c r="B99" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C99" s="6" t="s">
+      <c r="C99" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D99" s="2"/>
@@ -4734,13 +4736,13 @@
       <c r="Z99" s="2"/>
     </row>
     <row r="100" ht="14.25" customHeight="1">
-      <c r="A100" s="6" t="s">
+      <c r="A100" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B100" s="7" t="s">
+      <c r="B100" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C100" s="6" t="s">
+      <c r="C100" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D100" s="2"/>
@@ -4768,13 +4770,15 @@
       <c r="Z100" s="2"/>
     </row>
     <row r="101" ht="14.25" customHeight="1">
-      <c r="A101" s="6" t="s">
+      <c r="A101" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B101" s="6" t="s">
+      <c r="B101" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C101" s="8"/>
+      <c r="C101" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D101" s="2"/>
       <c r="E101" s="2"/>
       <c r="F101" s="2"/>
@@ -4800,13 +4804,15 @@
       <c r="Z101" s="2"/>
     </row>
     <row r="102" ht="14.25" customHeight="1">
-      <c r="A102" s="6" t="s">
+      <c r="A102" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B102" s="7" t="s">
+      <c r="B102" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C102" s="8"/>
+      <c r="C102" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
       <c r="F102" s="2"/>
@@ -4832,13 +4838,15 @@
       <c r="Z102" s="2"/>
     </row>
     <row r="103" ht="14.25" customHeight="1">
-      <c r="A103" s="6" t="s">
+      <c r="A103" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B103" s="7" t="s">
+      <c r="B103" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C103" s="8"/>
+      <c r="C103" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
       <c r="F103" s="2"/>
@@ -4864,13 +4872,15 @@
       <c r="Z103" s="2"/>
     </row>
     <row r="104" ht="14.25" customHeight="1">
-      <c r="A104" s="6" t="s">
+      <c r="A104" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B104" s="6" t="s">
+      <c r="B104" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C104" s="8"/>
+      <c r="C104" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D104" s="2"/>
       <c r="E104" s="2"/>
       <c r="F104" s="2"/>
@@ -4896,13 +4906,15 @@
       <c r="Z104" s="2"/>
     </row>
     <row r="105" ht="14.25" customHeight="1">
-      <c r="A105" s="6" t="s">
+      <c r="A105" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B105" s="7" t="s">
+      <c r="B105" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C105" s="8"/>
+      <c r="C105" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D105" s="2"/>
       <c r="E105" s="2"/>
       <c r="F105" s="2"/>
@@ -4928,9 +4940,9 @@
       <c r="Z105" s="2"/>
     </row>
     <row r="106" ht="14.25" customHeight="1">
-      <c r="A106" s="6"/>
-      <c r="B106" s="7"/>
-      <c r="C106" s="8"/>
+      <c r="A106" s="2"/>
+      <c r="B106" s="2"/>
+      <c r="C106" s="2"/>
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
       <c r="F106" s="2"/>
@@ -4956,9 +4968,15 @@
       <c r="Z106" s="2"/>
     </row>
     <row r="107" ht="14.25" customHeight="1">
-      <c r="A107" s="2"/>
-      <c r="B107" s="9"/>
-      <c r="C107" s="2"/>
+      <c r="A107" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D107" s="2"/>
       <c r="E107" s="2"/>
       <c r="F107" s="2"/>
@@ -4984,9 +5002,15 @@
       <c r="Z107" s="2"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
-      <c r="A108" s="2"/>
-      <c r="B108" s="2"/>
-      <c r="C108" s="2"/>
+      <c r="A108" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
       <c r="F108" s="2"/>
@@ -5012,9 +5036,15 @@
       <c r="Z108" s="2"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
-      <c r="A109" s="2"/>
-      <c r="B109" s="2"/>
-      <c r="C109" s="2"/>
+      <c r="A109" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D109" s="2"/>
       <c r="E109" s="2"/>
       <c r="F109" s="2"/>
@@ -5040,9 +5070,15 @@
       <c r="Z109" s="2"/>
     </row>
     <row r="110" ht="14.25" customHeight="1">
-      <c r="A110" s="2"/>
-      <c r="B110" s="2"/>
-      <c r="C110" s="2"/>
+      <c r="A110" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D110" s="2"/>
       <c r="E110" s="2"/>
       <c r="F110" s="2"/>
@@ -5068,9 +5104,15 @@
       <c r="Z110" s="2"/>
     </row>
     <row r="111" ht="14.25" customHeight="1">
-      <c r="A111" s="2"/>
-      <c r="B111" s="2"/>
-      <c r="C111" s="2"/>
+      <c r="A111" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D111" s="2"/>
       <c r="E111" s="2"/>
       <c r="F111" s="2"/>
@@ -5096,9 +5138,15 @@
       <c r="Z111" s="2"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
-      <c r="A112" s="2"/>
-      <c r="B112" s="2"/>
-      <c r="C112" s="2"/>
+      <c r="A112" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B112" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
       <c r="F112" s="2"/>
@@ -5124,9 +5172,15 @@
       <c r="Z112" s="2"/>
     </row>
     <row r="113" ht="14.25" customHeight="1">
-      <c r="A113" s="2"/>
-      <c r="B113" s="2"/>
-      <c r="C113" s="2"/>
+      <c r="A113" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D113" s="2"/>
       <c r="E113" s="2"/>
       <c r="F113" s="2"/>
@@ -5152,9 +5206,15 @@
       <c r="Z113" s="2"/>
     </row>
     <row r="114" ht="14.25" customHeight="1">
-      <c r="A114" s="2"/>
-      <c r="B114" s="2"/>
-      <c r="C114" s="2"/>
+      <c r="A114" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B114" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>114</v>
+      </c>
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
       <c r="F114" s="2"/>

</xml_diff>

<commit_message>
DP: start new future - join_forecast_bau_230711 - change paths
</commit_message>
<xml_diff>
--- a/create_forecast_basic/future/מיקום מקורי של הקבצים.xlsx
+++ b/create_forecast_basic/future/מיקום מקורי של הקבצים.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="146">
   <si>
     <t>שם קובץ</t>
   </si>
@@ -1161,6 +1161,96 @@
   <si>
     <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\iplan\join_forecast</t>
   </si>
+  <si>
+    <t>join_kibolt_2050_Jewish_bau_230712.ipynb</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\jew_kibolet\input</t>
+  </si>
+  <si>
+    <t>create_age_distribution_bau_230721.ipynb</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\jew_kibolet\output</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2020_2025_bau</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\jew_pop</t>
+  </si>
+  <si>
+    <t>230709_join_arab_jew_pop_bau.ipynb</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2025_2030_bau</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2030_2035_bau</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2035_2040_bau</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2040_2045_bau</t>
+  </si>
+  <si>
+    <t>230720_forecast_pop_jewish_2045_2050_bau</t>
+  </si>
+  <si>
+    <t>230720_pop_2025_bau</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\join_pop</t>
+  </si>
+  <si>
+    <t>change_pop_to_bau_goals_till_2050_230711.ipynb</t>
+  </si>
+  <si>
+    <t>230720_pop_2030_bau</t>
+  </si>
+  <si>
+    <t>230720_pop_2035_bau</t>
+  </si>
+  <si>
+    <t>230720_pop_2040_bau</t>
+  </si>
+  <si>
+    <t>230720_pop_2045_bau</t>
+  </si>
+  <si>
+    <t>230720_pop_2050_bau</t>
+  </si>
+  <si>
+    <t>gov_goals_2025_BAU</t>
+  </si>
+  <si>
+    <t>gov_goals_2030_BAU</t>
+  </si>
+  <si>
+    <t>gov_goals_2035_BAU</t>
+  </si>
+  <si>
+    <t>gov_goals_2040_BAU</t>
+  </si>
+  <si>
+    <t>gov_goals_2045_BAU</t>
+  </si>
+  <si>
+    <t>gov_goals_2050_BAU</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\change_pop</t>
+  </si>
+  <si>
+    <t>creat_forecast_2050_bau_230720.ipynb</t>
+  </si>
+  <si>
+    <t>join_forecast_bau_230711.ipynb</t>
+  </si>
+  <si>
+    <t>W:\Projects\הסעת המונים\01_שלב ה\קבצי עבודה\תחזיות_דמוגרפיות\תחזיות_2050\bau\join_forecast</t>
+  </si>
 </sst>
 </file>
 
@@ -1199,7 +1289,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1222,6 +1312,7 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -4968,13 +5059,13 @@
       <c r="Z106" s="2"/>
     </row>
     <row r="107" ht="14.25" customHeight="1">
-      <c r="A107" s="6" t="s">
+      <c r="A107" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B107" s="6" t="s">
+      <c r="B107" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C107" s="6" t="s">
+      <c r="C107" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D107" s="2"/>
@@ -5002,13 +5093,13 @@
       <c r="Z107" s="2"/>
     </row>
     <row r="108" ht="14.25" customHeight="1">
-      <c r="A108" s="6" t="s">
+      <c r="A108" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B108" s="7" t="s">
+      <c r="B108" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C108" s="6" t="s">
+      <c r="C108" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D108" s="2"/>
@@ -5036,13 +5127,13 @@
       <c r="Z108" s="2"/>
     </row>
     <row r="109" ht="14.25" customHeight="1">
-      <c r="A109" s="6" t="s">
+      <c r="A109" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B109" s="7" t="s">
+      <c r="B109" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C109" s="6" t="s">
+      <c r="C109" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D109" s="2"/>
@@ -5070,13 +5161,13 @@
       <c r="Z109" s="2"/>
     </row>
     <row r="110" ht="14.25" customHeight="1">
-      <c r="A110" s="6" t="s">
+      <c r="A110" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B110" s="7" t="s">
+      <c r="B110" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C110" s="6" t="s">
+      <c r="C110" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D110" s="2"/>
@@ -5104,13 +5195,13 @@
       <c r="Z110" s="2"/>
     </row>
     <row r="111" ht="14.25" customHeight="1">
-      <c r="A111" s="6" t="s">
+      <c r="A111" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B111" s="7" t="s">
+      <c r="B111" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C111" s="6" t="s">
+      <c r="C111" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D111" s="2"/>
@@ -5138,13 +5229,13 @@
       <c r="Z111" s="2"/>
     </row>
     <row r="112" ht="14.25" customHeight="1">
-      <c r="A112" s="6" t="s">
+      <c r="A112" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B112" s="7" t="s">
+      <c r="B112" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C112" s="6" t="s">
+      <c r="C112" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D112" s="2"/>
@@ -5172,13 +5263,13 @@
       <c r="Z112" s="2"/>
     </row>
     <row r="113" ht="14.25" customHeight="1">
-      <c r="A113" s="6" t="s">
+      <c r="A113" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B113" s="7" t="s">
+      <c r="B113" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C113" s="6" t="s">
+      <c r="C113" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D113" s="2"/>
@@ -5206,13 +5297,13 @@
       <c r="Z113" s="2"/>
     </row>
     <row r="114" ht="14.25" customHeight="1">
-      <c r="A114" s="6" t="s">
+      <c r="A114" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B114" s="7" t="s">
+      <c r="B114" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C114" s="6" t="s">
+      <c r="C114" s="2" t="s">
         <v>114</v>
       </c>
       <c r="D114" s="2"/>
@@ -5268,9 +5359,15 @@
       <c r="Z115" s="2"/>
     </row>
     <row r="116" ht="14.25" customHeight="1">
-      <c r="A116" s="2"/>
-      <c r="B116" s="2"/>
-      <c r="C116" s="2"/>
+      <c r="A116" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B116" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
       <c r="F116" s="2"/>
@@ -5296,9 +5393,15 @@
       <c r="Z116" s="2"/>
     </row>
     <row r="117" ht="14.25" customHeight="1">
-      <c r="A117" s="2"/>
-      <c r="B117" s="2"/>
-      <c r="C117" s="2"/>
+      <c r="A117" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D117" s="2"/>
       <c r="E117" s="2"/>
       <c r="F117" s="2"/>
@@ -5324,9 +5427,15 @@
       <c r="Z117" s="2"/>
     </row>
     <row r="118" ht="14.25" customHeight="1">
-      <c r="A118" s="2"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="2"/>
+      <c r="A118" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
       <c r="F118" s="2"/>
@@ -5352,9 +5461,15 @@
       <c r="Z118" s="2"/>
     </row>
     <row r="119" ht="14.25" customHeight="1">
-      <c r="A119" s="2"/>
-      <c r="B119" s="2"/>
-      <c r="C119" s="2"/>
+      <c r="A119" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
       <c r="F119" s="2"/>
@@ -5380,9 +5495,15 @@
       <c r="Z119" s="2"/>
     </row>
     <row r="120" ht="14.25" customHeight="1">
-      <c r="A120" s="2"/>
-      <c r="B120" s="2"/>
-      <c r="C120" s="2"/>
+      <c r="A120" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B120" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D120" s="2"/>
       <c r="E120" s="2"/>
       <c r="F120" s="2"/>
@@ -5408,9 +5529,15 @@
       <c r="Z120" s="2"/>
     </row>
     <row r="121" ht="14.25" customHeight="1">
-      <c r="A121" s="2"/>
-      <c r="B121" s="2"/>
-      <c r="C121" s="2"/>
+      <c r="A121" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B121" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>116</v>
+      </c>
       <c r="D121" s="2"/>
       <c r="E121" s="2"/>
       <c r="F121" s="2"/>
@@ -5464,9 +5591,15 @@
       <c r="Z122" s="2"/>
     </row>
     <row r="123" ht="14.25" customHeight="1">
-      <c r="A123" s="2"/>
-      <c r="B123" s="2"/>
-      <c r="C123" s="2"/>
+      <c r="A123" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C123" s="6" t="s">
+        <v>118</v>
+      </c>
       <c r="D123" s="2"/>
       <c r="E123" s="2"/>
       <c r="F123" s="2"/>
@@ -5492,9 +5625,15 @@
       <c r="Z123" s="2"/>
     </row>
     <row r="124" ht="14.25" customHeight="1">
-      <c r="A124" s="2"/>
-      <c r="B124" s="2"/>
-      <c r="C124" s="2"/>
+      <c r="A124" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B124" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C124" s="6" t="s">
+        <v>118</v>
+      </c>
       <c r="D124" s="2"/>
       <c r="E124" s="2"/>
       <c r="F124" s="2"/>
@@ -5520,9 +5659,15 @@
       <c r="Z124" s="2"/>
     </row>
     <row r="125" ht="14.25" customHeight="1">
-      <c r="A125" s="2"/>
-      <c r="B125" s="2"/>
-      <c r="C125" s="2"/>
+      <c r="A125" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B125" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C125" s="6" t="s">
+        <v>118</v>
+      </c>
       <c r="D125" s="2"/>
       <c r="E125" s="2"/>
       <c r="F125" s="2"/>
@@ -5548,9 +5693,15 @@
       <c r="Z125" s="2"/>
     </row>
     <row r="126" ht="14.25" customHeight="1">
-      <c r="A126" s="2"/>
-      <c r="B126" s="2"/>
-      <c r="C126" s="2"/>
+      <c r="A126" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B126" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C126" s="6" t="s">
+        <v>118</v>
+      </c>
       <c r="D126" s="2"/>
       <c r="E126" s="2"/>
       <c r="F126" s="2"/>
@@ -5604,9 +5755,15 @@
       <c r="Z127" s="2"/>
     </row>
     <row r="128" ht="14.25" customHeight="1">
-      <c r="A128" s="2"/>
-      <c r="B128" s="2"/>
-      <c r="C128" s="2"/>
+      <c r="A128" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B128" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C128" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D128" s="2"/>
       <c r="E128" s="2"/>
       <c r="F128" s="2"/>
@@ -5632,9 +5789,15 @@
       <c r="Z128" s="2"/>
     </row>
     <row r="129" ht="14.25" customHeight="1">
-      <c r="A129" s="2"/>
-      <c r="B129" s="2"/>
-      <c r="C129" s="2"/>
+      <c r="A129" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B129" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C129" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
       <c r="F129" s="2"/>
@@ -5660,9 +5823,15 @@
       <c r="Z129" s="2"/>
     </row>
     <row r="130" ht="14.25" customHeight="1">
-      <c r="A130" s="2"/>
-      <c r="B130" s="2"/>
-      <c r="C130" s="2"/>
+      <c r="A130" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B130" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C130" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
       <c r="F130" s="2"/>
@@ -5688,9 +5857,15 @@
       <c r="Z130" s="2"/>
     </row>
     <row r="131" ht="14.25" customHeight="1">
-      <c r="A131" s="2"/>
-      <c r="B131" s="2"/>
-      <c r="C131" s="2"/>
+      <c r="A131" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C131" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
       <c r="F131" s="2"/>
@@ -5716,9 +5891,15 @@
       <c r="Z131" s="2"/>
     </row>
     <row r="132" ht="14.25" customHeight="1">
-      <c r="A132" s="2"/>
-      <c r="B132" s="2"/>
-      <c r="C132" s="2"/>
+      <c r="A132" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B132" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C132" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
       <c r="F132" s="2"/>
@@ -5744,9 +5925,15 @@
       <c r="Z132" s="2"/>
     </row>
     <row r="133" ht="14.25" customHeight="1">
-      <c r="A133" s="2"/>
-      <c r="B133" s="2"/>
-      <c r="C133" s="2"/>
+      <c r="A133" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B133" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C133" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D133" s="2"/>
       <c r="E133" s="2"/>
       <c r="F133" s="2"/>
@@ -5772,9 +5959,15 @@
       <c r="Z133" s="2"/>
     </row>
     <row r="134" ht="14.25" customHeight="1">
-      <c r="A134" s="2"/>
-      <c r="B134" s="2"/>
-      <c r="C134" s="2"/>
+      <c r="A134" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B134" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C134" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D134" s="2"/>
       <c r="E134" s="2"/>
       <c r="F134" s="2"/>
@@ -5800,9 +5993,15 @@
       <c r="Z134" s="2"/>
     </row>
     <row r="135" ht="14.25" customHeight="1">
-      <c r="A135" s="2"/>
-      <c r="B135" s="2"/>
-      <c r="C135" s="2"/>
+      <c r="A135" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C135" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D135" s="2"/>
       <c r="E135" s="2"/>
       <c r="F135" s="2"/>
@@ -5828,9 +6027,15 @@
       <c r="Z135" s="2"/>
     </row>
     <row r="136" ht="14.25" customHeight="1">
-      <c r="A136" s="2"/>
-      <c r="B136" s="2"/>
-      <c r="C136" s="2"/>
+      <c r="A136" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B136" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C136" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D136" s="2"/>
       <c r="E136" s="2"/>
       <c r="F136" s="2"/>
@@ -5856,9 +6061,15 @@
       <c r="Z136" s="2"/>
     </row>
     <row r="137" ht="14.25" customHeight="1">
-      <c r="A137" s="2"/>
-      <c r="B137" s="2"/>
-      <c r="C137" s="2"/>
+      <c r="A137" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C137" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D137" s="2"/>
       <c r="E137" s="2"/>
       <c r="F137" s="2"/>
@@ -5884,9 +6095,15 @@
       <c r="Z137" s="2"/>
     </row>
     <row r="138" ht="14.25" customHeight="1">
-      <c r="A138" s="2"/>
-      <c r="B138" s="2"/>
-      <c r="C138" s="2"/>
+      <c r="A138" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B138" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C138" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D138" s="2"/>
       <c r="E138" s="2"/>
       <c r="F138" s="2"/>
@@ -5912,9 +6129,15 @@
       <c r="Z138" s="2"/>
     </row>
     <row r="139" ht="14.25" customHeight="1">
-      <c r="A139" s="2"/>
-      <c r="B139" s="2"/>
-      <c r="C139" s="2"/>
+      <c r="A139" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B139" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C139" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="D139" s="2"/>
       <c r="E139" s="2"/>
       <c r="F139" s="2"/>
@@ -5968,9 +6191,15 @@
       <c r="Z140" s="2"/>
     </row>
     <row r="141" ht="14.25" customHeight="1">
-      <c r="A141" s="2"/>
-      <c r="B141" s="2"/>
-      <c r="C141" s="2"/>
+      <c r="A141" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C141" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D141" s="2"/>
       <c r="E141" s="2"/>
       <c r="F141" s="2"/>
@@ -5996,9 +6225,15 @@
       <c r="Z141" s="2"/>
     </row>
     <row r="142" ht="14.25" customHeight="1">
-      <c r="A142" s="2"/>
-      <c r="B142" s="2"/>
-      <c r="C142" s="2"/>
+      <c r="A142" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B142" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C142" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D142" s="2"/>
       <c r="E142" s="2"/>
       <c r="F142" s="2"/>
@@ -6024,9 +6259,15 @@
       <c r="Z142" s="2"/>
     </row>
     <row r="143" ht="14.25" customHeight="1">
-      <c r="A143" s="2"/>
-      <c r="B143" s="2"/>
-      <c r="C143" s="2"/>
+      <c r="A143" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C143" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D143" s="2"/>
       <c r="E143" s="2"/>
       <c r="F143" s="2"/>
@@ -6052,9 +6293,15 @@
       <c r="Z143" s="2"/>
     </row>
     <row r="144" ht="14.25" customHeight="1">
-      <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
+      <c r="A144" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B144" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C144" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D144" s="2"/>
       <c r="E144" s="2"/>
       <c r="F144" s="2"/>
@@ -6080,9 +6327,15 @@
       <c r="Z144" s="2"/>
     </row>
     <row r="145" ht="14.25" customHeight="1">
-      <c r="A145" s="2"/>
-      <c r="B145" s="2"/>
-      <c r="C145" s="2"/>
+      <c r="A145" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B145" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C145" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D145" s="2"/>
       <c r="E145" s="2"/>
       <c r="F145" s="2"/>
@@ -6108,9 +6361,15 @@
       <c r="Z145" s="2"/>
     </row>
     <row r="146" ht="14.25" customHeight="1">
-      <c r="A146" s="2"/>
-      <c r="B146" s="2"/>
-      <c r="C146" s="2"/>
+      <c r="A146" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B146" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D146" s="2"/>
       <c r="E146" s="2"/>
       <c r="F146" s="2"/>
@@ -6136,9 +6395,15 @@
       <c r="Z146" s="2"/>
     </row>
     <row r="147" ht="14.25" customHeight="1">
-      <c r="A147" s="2"/>
-      <c r="B147" s="2"/>
-      <c r="C147" s="2"/>
+      <c r="A147" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C147" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D147" s="2"/>
       <c r="E147" s="2"/>
       <c r="F147" s="2"/>
@@ -6164,9 +6429,15 @@
       <c r="Z147" s="2"/>
     </row>
     <row r="148" ht="14.25" customHeight="1">
-      <c r="A148" s="2"/>
-      <c r="B148" s="2"/>
-      <c r="C148" s="2"/>
+      <c r="A148" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B148" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C148" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D148" s="2"/>
       <c r="E148" s="2"/>
       <c r="F148" s="2"/>
@@ -6192,9 +6463,15 @@
       <c r="Z148" s="2"/>
     </row>
     <row r="149" ht="14.25" customHeight="1">
-      <c r="A149" s="2"/>
-      <c r="B149" s="2"/>
-      <c r="C149" s="2"/>
+      <c r="A149" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C149" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D149" s="2"/>
       <c r="E149" s="2"/>
       <c r="F149" s="2"/>
@@ -6220,9 +6497,15 @@
       <c r="Z149" s="2"/>
     </row>
     <row r="150" ht="14.25" customHeight="1">
-      <c r="A150" s="2"/>
-      <c r="B150" s="2"/>
-      <c r="C150" s="2"/>
+      <c r="A150" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C150" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
       <c r="F150" s="2"/>
@@ -6248,9 +6531,15 @@
       <c r="Z150" s="2"/>
     </row>
     <row r="151" ht="14.25" customHeight="1">
-      <c r="A151" s="2"/>
-      <c r="B151" s="2"/>
-      <c r="C151" s="2"/>
+      <c r="A151" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C151" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
       <c r="F151" s="2"/>
@@ -6276,9 +6565,15 @@
       <c r="Z151" s="2"/>
     </row>
     <row r="152" ht="14.25" customHeight="1">
-      <c r="A152" s="2"/>
-      <c r="B152" s="2"/>
-      <c r="C152" s="2"/>
+      <c r="A152" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B152" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C152" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
       <c r="F152" s="2"/>
@@ -6304,9 +6599,15 @@
       <c r="Z152" s="2"/>
     </row>
     <row r="153" ht="14.25" customHeight="1">
-      <c r="A153" s="2"/>
-      <c r="B153" s="2"/>
-      <c r="C153" s="2"/>
+      <c r="A153" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C153" s="6" t="s">
+        <v>130</v>
+      </c>
       <c r="D153" s="2"/>
       <c r="E153" s="2"/>
       <c r="F153" s="2"/>
@@ -6360,9 +6661,15 @@
       <c r="Z154" s="2"/>
     </row>
     <row r="155" ht="14.25" customHeight="1">
-      <c r="A155" s="2"/>
-      <c r="B155" s="2"/>
-      <c r="C155" s="2"/>
+      <c r="A155" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C155" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
       <c r="F155" s="2"/>
@@ -6388,9 +6695,15 @@
       <c r="Z155" s="2"/>
     </row>
     <row r="156" ht="14.25" customHeight="1">
-      <c r="A156" s="2"/>
-      <c r="B156" s="2"/>
-      <c r="C156" s="2"/>
+      <c r="A156" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C156" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
       <c r="F156" s="2"/>
@@ -6416,9 +6729,15 @@
       <c r="Z156" s="2"/>
     </row>
     <row r="157" ht="14.25" customHeight="1">
-      <c r="A157" s="2"/>
-      <c r="B157" s="2"/>
-      <c r="C157" s="2"/>
+      <c r="A157" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C157" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
       <c r="F157" s="2"/>
@@ -6444,9 +6763,15 @@
       <c r="Z157" s="2"/>
     </row>
     <row r="158" ht="14.25" customHeight="1">
-      <c r="A158" s="2"/>
-      <c r="B158" s="2"/>
-      <c r="C158" s="2"/>
+      <c r="A158" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B158" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C158" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
       <c r="F158" s="2"/>
@@ -6472,9 +6797,15 @@
       <c r="Z158" s="2"/>
     </row>
     <row r="159" ht="14.25" customHeight="1">
-      <c r="A159" s="2"/>
-      <c r="B159" s="2"/>
-      <c r="C159" s="2"/>
+      <c r="A159" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C159" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D159" s="2"/>
       <c r="E159" s="2"/>
       <c r="F159" s="2"/>
@@ -6500,9 +6831,15 @@
       <c r="Z159" s="2"/>
     </row>
     <row r="160" ht="14.25" customHeight="1">
-      <c r="A160" s="2"/>
-      <c r="B160" s="2"/>
-      <c r="C160" s="2"/>
+      <c r="A160" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B160" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C160" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D160" s="2"/>
       <c r="E160" s="2"/>
       <c r="F160" s="2"/>
@@ -6528,9 +6865,15 @@
       <c r="Z160" s="2"/>
     </row>
     <row r="161" ht="14.25" customHeight="1">
-      <c r="A161" s="2"/>
-      <c r="B161" s="2"/>
-      <c r="C161" s="2"/>
+      <c r="A161" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C161" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D161" s="2"/>
       <c r="E161" s="2"/>
       <c r="F161" s="2"/>
@@ -6556,9 +6899,15 @@
       <c r="Z161" s="2"/>
     </row>
     <row r="162" ht="14.25" customHeight="1">
-      <c r="A162" s="2"/>
-      <c r="B162" s="2"/>
-      <c r="C162" s="2"/>
+      <c r="A162" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B162" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C162" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
       <c r="F162" s="2"/>
@@ -6584,9 +6933,15 @@
       <c r="Z162" s="2"/>
     </row>
     <row r="163" ht="14.25" customHeight="1">
-      <c r="A163" s="2"/>
-      <c r="B163" s="2"/>
-      <c r="C163" s="2"/>
+      <c r="A163" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B163" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C163" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D163" s="2"/>
       <c r="E163" s="2"/>
       <c r="F163" s="2"/>
@@ -6612,9 +6967,15 @@
       <c r="Z163" s="2"/>
     </row>
     <row r="164" ht="14.25" customHeight="1">
-      <c r="A164" s="2"/>
-      <c r="B164" s="2"/>
-      <c r="C164" s="2"/>
+      <c r="A164" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B164" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C164" s="6" t="s">
+        <v>143</v>
+      </c>
       <c r="D164" s="2"/>
       <c r="E164" s="2"/>
       <c r="F164" s="2"/>
@@ -6640,9 +7001,9 @@
       <c r="Z164" s="2"/>
     </row>
     <row r="165" ht="14.25" customHeight="1">
-      <c r="A165" s="2"/>
-      <c r="B165" s="2"/>
-      <c r="C165" s="2"/>
+      <c r="A165" s="6"/>
+      <c r="B165" s="7"/>
+      <c r="C165" s="8"/>
       <c r="D165" s="2"/>
       <c r="E165" s="2"/>
       <c r="F165" s="2"/>
@@ -6668,9 +7029,15 @@
       <c r="Z165" s="2"/>
     </row>
     <row r="166" ht="14.25" customHeight="1">
-      <c r="A166" s="2"/>
-      <c r="B166" s="2"/>
-      <c r="C166" s="2"/>
+      <c r="A166" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B166" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C166" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
       <c r="F166" s="2"/>
@@ -6696,9 +7063,15 @@
       <c r="Z166" s="2"/>
     </row>
     <row r="167" ht="14.25" customHeight="1">
-      <c r="A167" s="2"/>
-      <c r="B167" s="2"/>
-      <c r="C167" s="2"/>
+      <c r="A167" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C167" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D167" s="2"/>
       <c r="E167" s="2"/>
       <c r="F167" s="2"/>
@@ -6724,9 +7097,15 @@
       <c r="Z167" s="2"/>
     </row>
     <row r="168" ht="14.25" customHeight="1">
-      <c r="A168" s="2"/>
-      <c r="B168" s="2"/>
-      <c r="C168" s="2"/>
+      <c r="A168" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B168" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C168" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
       <c r="F168" s="2"/>
@@ -6752,9 +7131,15 @@
       <c r="Z168" s="2"/>
     </row>
     <row r="169" ht="14.25" customHeight="1">
-      <c r="A169" s="2"/>
-      <c r="B169" s="2"/>
-      <c r="C169" s="2"/>
+      <c r="A169" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C169" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
       <c r="F169" s="2"/>
@@ -6780,9 +7165,15 @@
       <c r="Z169" s="2"/>
     </row>
     <row r="170" ht="14.25" customHeight="1">
-      <c r="A170" s="2"/>
-      <c r="B170" s="2"/>
-      <c r="C170" s="2"/>
+      <c r="A170" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B170" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C170" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
       <c r="F170" s="2"/>
@@ -6808,9 +7199,15 @@
       <c r="Z170" s="2"/>
     </row>
     <row r="171" ht="14.25" customHeight="1">
-      <c r="A171" s="2"/>
-      <c r="B171" s="2"/>
-      <c r="C171" s="2"/>
+      <c r="A171" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C171" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D171" s="2"/>
       <c r="E171" s="2"/>
       <c r="F171" s="2"/>
@@ -6836,9 +7233,15 @@
       <c r="Z171" s="2"/>
     </row>
     <row r="172" ht="14.25" customHeight="1">
-      <c r="A172" s="2"/>
-      <c r="B172" s="2"/>
-      <c r="C172" s="2"/>
+      <c r="A172" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C172" s="6" t="s">
+        <v>144</v>
+      </c>
       <c r="D172" s="2"/>
       <c r="E172" s="2"/>
       <c r="F172" s="2"/>
@@ -6864,9 +7267,13 @@
       <c r="Z172" s="2"/>
     </row>
     <row r="173" ht="14.25" customHeight="1">
-      <c r="A173" s="2"/>
-      <c r="B173" s="2"/>
-      <c r="C173" s="2"/>
+      <c r="A173" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C173" s="8"/>
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
       <c r="F173" s="2"/>

</xml_diff>